<commit_message>
Update Catan data files and enhance visualization scripts
- Updated raw data files: Catan_RawData_Copy.xlsx and Catan_RawData_Original.xlsx
- Added new histogram graph: Catan_Histogram_Iedereenlos.png
- Updated existing graph: Catan_TotaleScores_Alles.png
- Added new graph without dates: Catan_TotaleScores_Alles_ZonderDatum.png
- Introduced new pie chart: Piechart_Begon_Bank.png
- Expanded ToDo list with additional tasks for scoring and visualization improvements
- Enhanced Jupyter notebook with new histogram plotting code and error handling
</commit_message>
<xml_diff>
--- a/Data/Excel/Catan_RawData_Copy.xlsx
+++ b/Data/Excel/Catan_RawData_Copy.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30404"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{85D7B749-9812-4081-A96E-5A39500D9782}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B2E40174-3AD8-4066-9B03-741D2A8B4536}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="30">
   <si>
     <t>Datum</t>
   </si>
@@ -94,9 +94,6 @@
   </si>
   <si>
     <t>Terschelling</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ma </t>
   </si>
   <si>
     <t>1ste paasdag</t>
@@ -1710,13 +1707,13 @@
         <v>11</v>
       </c>
       <c r="G39" t="s">
+        <v>4</v>
+      </c>
+      <c r="H39" t="s">
+        <v>4</v>
+      </c>
+      <c r="I39" t="s">
         <v>20</v>
-      </c>
-      <c r="H39" t="s">
-        <v>4</v>
-      </c>
-      <c r="I39" t="s">
-        <v>21</v>
       </c>
       <c r="J39">
         <v>38</v>
@@ -1751,7 +1748,7 @@
         <v>4</v>
       </c>
       <c r="I40" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="J40">
         <v>39</v>
@@ -1818,7 +1815,7 @@
         <v>4</v>
       </c>
       <c r="I42" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="J42">
         <v>41</v>
@@ -1853,7 +1850,7 @@
         <v>5</v>
       </c>
       <c r="I43" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J43">
         <v>42</v>
@@ -1952,7 +1949,7 @@
         <v>5</v>
       </c>
       <c r="I46" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="J46">
         <v>45</v>
@@ -2083,7 +2080,7 @@
         <v>4</v>
       </c>
       <c r="I50" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J50">
         <v>49</v>
@@ -2310,7 +2307,7 @@
         <v>3</v>
       </c>
       <c r="I57" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="J57">
         <v>56</v>
@@ -2409,7 +2406,7 @@
         <v>1</v>
       </c>
       <c r="I60" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="J60">
         <v>59</v>
@@ -2767,7 +2764,7 @@
         <v>4</v>
       </c>
       <c r="I71" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="J71">
         <v>70</v>
@@ -2802,7 +2799,7 @@
         <v>4</v>
       </c>
       <c r="I72" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="J72">
         <v>71</v>
@@ -2869,7 +2866,7 @@
         <v>4</v>
       </c>
       <c r="I74" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="J74">
         <v>73</v>
@@ -2904,7 +2901,7 @@
         <v>4</v>
       </c>
       <c r="I75" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="J75">
         <v>74</v>
@@ -2939,7 +2936,7 @@
         <v>1</v>
       </c>
       <c r="I76" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="J76">
         <v>75</v>

</xml_diff>